<commit_message>
Update US WDSI data
</commit_message>
<xml_diff>
--- a/data/AU.xlsx
+++ b/data/AU.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1400"/>
+  <dimension ref="A1:E1401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25112,6 +25112,23 @@
         <v>0.06666666666666667</v>
       </c>
       <c r="E1400" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr"/>
+      <c r="C1401" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1401" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1401" t="b">
         <v>0</v>
       </c>
     </row>
@@ -25145,7 +25162,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Coverage: 2022-05-25 to 2026-03-23 | Publication days: 471</t>
+          <t>Coverage: 2022-05-25 to 2026-03-24 | Publication days: 471</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update US data from local refresh
</commit_message>
<xml_diff>
--- a/data/AU.xlsx
+++ b/data/AU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="daily_data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="variable_definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="variable_definitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -42,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,14 +53,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,27 +446,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>raw</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>rolling7</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>rolling30</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
@@ -25172,21 +25184,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Australia WDSI Data Workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Coverage: 2022-05-25 to 2026-03-25 | Publication days: 472</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Locked to DSI-ICF/code/data_integration.executed.ipynb: publication-day raw score = same-day minimum, then forward-fill missing days, then compute rolling means on the filled daily path.</t>
         </is>
@@ -25194,22 +25206,22 @@
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>units_or_scale</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>

</xml_diff>

<commit_message>
Deepen local US reclassification refresh
</commit_message>
<xml_diff>
--- a/data/AU.xlsx
+++ b/data/AU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="daily_data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="variable_definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="variable_definitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -42,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,14 +53,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,27 +446,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>raw</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>rolling7</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>rolling30</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
@@ -25189,21 +25201,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Australia WDSI Data Workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Coverage: 2022-05-25 to 2026-03-26 | Publication days: 472</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Locked to DSI-ICF/code/data_integration.executed.ipynb: publication-day raw score = same-day minimum, then forward-fill missing days, then compute rolling means on the filled daily path.</t>
         </is>
@@ -25211,22 +25223,22 @@
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>units_or_scale</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>

</xml_diff>

<commit_message>
Finish local US cleanup
</commit_message>
<xml_diff>
--- a/data/AU.xlsx
+++ b/data/AU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="daily_data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="variable_definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="daily_data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="variable_definitions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -42,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,14 +53,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,27 +446,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>raw</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>rolling7</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>rolling30</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>publication</t>
         </is>
@@ -25189,21 +25201,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Australia WDSI Data Workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Coverage: 2022-05-25 to 2026-03-26 | Publication days: 472</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Locked to DSI-ICF/code/data_integration.executed.ipynb: publication-day raw score = same-day minimum, then forward-fill missing days, then compute rolling means on the filled daily path.</t>
         </is>
@@ -25211,22 +25223,22 @@
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>variable</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>units_or_scale</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>

</xml_diff>